<commit_message>
Mindbody transform: past classes, visits and PT as Mindbody recorded them (#219)
- Download and read Cancellations "Group cancellations". A past class with no
  visits and no payroll line that it lists comes across cancelled, not Unpriced.
- Visit state comes from Late Cancel / No-show, and the roster's Status where
  the flags say neither. Staff Paid is ignored. An "unpaid" visit is attended
  with no package.
- Past PT keeps the roster's end time (an hour only as a counted fallback), its
  Appointment Notes as the request message, and the roster's "Scheduled by" as
  scheduled-by when that staff member comes across (else the owner, counted).
- A past PT no-show's request ends where the platform's own job leaves one, so
  no job moves it. A late-cancelled PT session is cancelled. A session paid
  from a 2on1 package has two places.
- Classes a substitute taught are counted in the preflight (no cover field).
</commit_message>
<xml_diff>
--- a/be/tools/mindbody/transform/fixtures/reports/Clients/16 Attendance/16 Attendance - Date - 2026.xlsx
+++ b/be/tools/mindbody/transform/fixtures/reports/Clients/16 Attendance/16 Attendance - Date - 2026.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -179,6 +179,27 @@
   </si>
   <si>
     <t xml:space="preserve">Signed in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT - Bundle of 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal Training / PT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner, Olive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main Hall </t>
+  </si>
+  <si>
+    <t xml:space="preserve">林, Mei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100000008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Show</t>
   </si>
   <si>
     <t xml:space="preserve">PT - Bundle of 10</t>
@@ -574,13 +595,13 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="B8">
-        <v>0.7916666666666666</v>
+        <v>0.375</v>
       </c>
       <c r="C8">
-        <v>0.8333333333333334</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="D8" t="s">
         <v>58</v>
@@ -588,98 +609,95 @@
       <c r="E8" t="s">
         <v>59</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>60</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>61</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>62</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>63</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>64</v>
-      </c>
-      <c r="K8" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B9">
-        <v>0.4166666666666667</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="C9">
-        <v>0.4583333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="D9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" t="s">
         <v>66</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>67</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>68</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>69</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>70</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>71</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>72</v>
-      </c>
-      <c r="K9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>46275</v>
+        <v>46273</v>
       </c>
       <c r="B10">
-        <v>0.7916666666666666</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="C10">
-        <v>0.8333333333333334</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="D10" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" t="s">
         <v>74</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>75</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>76</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>78</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>79</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>80</v>
-      </c>
-      <c r="K10" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="B11">
         <v>0.7916666666666666</v>
@@ -688,71 +706,74 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="D11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" t="s">
         <v>82</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>83</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>84</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>85</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>87</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>88</v>
-      </c>
-      <c r="K11" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B12">
-        <v>0.4166666666666667</v>
+        <v>0.7916666666666666</v>
       </c>
       <c r="C12">
-        <v>0.4583333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="D12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" t="s">
         <v>90</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>91</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>92</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>93</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>94</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>95</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>69400</v>
+        <v>46280</v>
       </c>
       <c r="B13">
-        <v>0.7916666666666666</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="C13">
-        <v>0.8333333333333334</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="D13" t="s">
         <v>97</v>
@@ -775,8 +796,40 @@
       <c r="J13" t="s">
         <v>103</v>
       </c>
-      <c r="K13" t="s">
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>69400</v>
+      </c>
+      <c r="B14">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="C14">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="D14" t="s">
         <v>104</v>
+      </c>
+      <c r="E14" t="s">
+        <v>105</v>
+      </c>
+      <c r="F14" t="s">
+        <v>106</v>
+      </c>
+      <c r="G14" t="s">
+        <v>107</v>
+      </c>
+      <c r="H14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I14" t="s">
+        <v>109</v>
+      </c>
+      <c r="J14" t="s">
+        <v>110</v>
+      </c>
+      <c r="K14" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>